<commit_message>
Se agregó el método limpiarCuentas
</commit_message>
<xml_diff>
--- a/public/PresupuestoInicial/presupuesto ingresos 2024.xlsx
+++ b/public/PresupuestoInicial/presupuesto ingresos 2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gustavor/Documents/Github/SAC-IPE/public/PresupuestoInicial/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\PresupuestoInicial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774C25FC-C77F-004F-B45D-05F7373D5481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00891D7-EE5C-45E3-A995-F7E969F88A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15200" yWindow="1380" windowWidth="14020" windowHeight="15580" tabRatio="822" xr2:uid="{9539A8D9-1841-4346-A922-0009B4A42F3E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="822" xr2:uid="{9539A8D9-1841-4346-A922-0009B4A42F3E}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato de carga ppto" sheetId="2" r:id="rId1"/>
@@ -474,9 +474,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -514,7 +514,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -620,7 +620,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -762,7 +762,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -771,21 +771,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E34018DD-ECDB-49CC-B8B4-8192DBA1B262}">
   <dimension ref="A1:T23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="51.6640625" style="12" customWidth="1"/>
-    <col min="7" max="7" width="26.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="20" width="14.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="21" max="16384" width="11.5" style="5"/>
+    <col min="3" max="3" width="11.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="51.7109375" style="12" customWidth="1"/>
+    <col min="7" max="7" width="26.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="20" width="14.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -847,7 +847,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>19</v>
       </c>
@@ -910,7 +910,7 @@
         <v>78493723.840000004</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
@@ -973,7 +973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>130822872.73999999</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="7" customFormat="1" ht="28" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" s="7" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>19</v>
       </c>
@@ -1162,7 +1162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>35</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>38</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>5450</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>41</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>41</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>2134560</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>46</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>49</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>27754.15</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>52</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>32</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>1331.33</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>57</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>46580371.969999999</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>60</v>
       </c>
@@ -1855,7 +1855,7 @@
         <v>982007.1</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>63</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>66</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>66</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>333333748</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>66</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>28654113</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>32</v>
       </c>
@@ -2170,7 +2170,7 @@
         <v>8583334</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="H23" s="13">
         <f>SUM(H2:H22)</f>
         <v>10965299525</v>

</xml_diff>